<commit_message>
mind PV voltage drom while high power generation switch solar production on only if produce
</commit_message>
<xml_diff>
--- a/references/PH1800 PV1800 EP1800 PV3500 EP3500 RS485 Modbud RTU communication Protocol 1.4.15.xlsx
+++ b/references/PH1800 PV1800 EP1800 PV3500 EP3500 RS485 Modbud RTU communication Protocol 1.4.15.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28129"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="28429"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ikost\source\repos\home-inverter-grafana-monitor\references\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8117F35-C913-4D00-8B2D-A44AF267A0FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92DA1195-808E-4A25-AC51-A11A3F49C1B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="483" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" tabRatio="483" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="hidden" r:id="rId1"/>
@@ -3390,9 +3390,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AB59"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="3" max="10" width="4.625" style="70" customWidth="1"/>
+    <col min="3" max="10" width="4.6640625" style="70" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10">
@@ -4775,7 +4775,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <sheetData/>
   <phoneticPr fontId="41" type="noConversion"/>
   <pageMargins left="0.69930555555555596" right="0.69930555555555596" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -4785,14 +4785,14 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:F164"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="17.25" customWidth="1"/>
-    <col min="2" max="2" width="22.625" customWidth="1"/>
-    <col min="3" max="3" width="36.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.21875" customWidth="1"/>
+    <col min="2" max="2" width="22.6640625" customWidth="1"/>
+    <col min="3" max="3" width="36.6640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31" customWidth="1"/>
-    <col min="5" max="5" width="27.625" customWidth="1"/>
-    <col min="6" max="6" width="65.75" customWidth="1"/>
+    <col min="5" max="5" width="27.6640625" customWidth="1"/>
+    <col min="6" max="6" width="65.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="55.5" customHeight="1">
@@ -5179,7 +5179,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="24" spans="1:6" s="39" customFormat="1" ht="72.95" customHeight="1">
+    <row r="24" spans="1:6" s="39" customFormat="1" ht="72.900000000000006" customHeight="1">
       <c r="A24" s="48">
         <v>20109</v>
       </c>
@@ -5453,7 +5453,7 @@
       </c>
       <c r="F39" s="53"/>
     </row>
-    <row r="40" spans="1:6" s="39" customFormat="1" ht="107.25" customHeight="1">
+    <row r="40" spans="1:6" s="39" customFormat="1" ht="138">
       <c r="A40" s="48">
         <v>20143</v>
       </c>
@@ -5503,7 +5503,7 @@
       </c>
       <c r="F42" s="19"/>
     </row>
-    <row r="43" spans="1:6" s="40" customFormat="1" ht="25.5">
+    <row r="43" spans="1:6" s="40" customFormat="1" ht="27.6">
       <c r="A43" s="96">
         <v>20214</v>
       </c>
@@ -6497,7 +6497,7 @@
       <c r="E105" s="96"/>
       <c r="F105" s="19"/>
     </row>
-    <row r="106" spans="1:6">
+    <row r="106" spans="1:6" ht="24">
       <c r="A106" s="43">
         <v>25261</v>
       </c>
@@ -6513,7 +6513,7 @@
       </c>
       <c r="F106" s="19"/>
     </row>
-    <row r="107" spans="1:6">
+    <row r="107" spans="1:6" ht="24">
       <c r="A107" s="43">
         <v>25262</v>
       </c>
@@ -6529,7 +6529,7 @@
       </c>
       <c r="F107" s="19"/>
     </row>
-    <row r="108" spans="1:6">
+    <row r="108" spans="1:6" ht="24">
       <c r="A108" s="43">
         <v>25263</v>
       </c>
@@ -6830,7 +6830,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="133" spans="1:3" ht="27">
+    <row r="133" spans="1:3" ht="28.8">
       <c r="A133" s="66">
         <v>3</v>
       </c>
@@ -6838,7 +6838,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="134" spans="1:3" ht="27">
+    <row r="134" spans="1:3" ht="28.8">
       <c r="A134" s="66">
         <v>4</v>
       </c>
@@ -6846,7 +6846,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="135" spans="1:3" ht="27">
+    <row r="135" spans="1:3" ht="28.8">
       <c r="A135" s="66">
         <v>5</v>
       </c>
@@ -6950,7 +6950,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="149" spans="1:3" ht="27">
+    <row r="149" spans="1:3" ht="28.8">
       <c r="A149" s="66">
         <v>0</v>
       </c>
@@ -6961,7 +6961,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="150" spans="1:3" ht="27">
+    <row r="150" spans="1:3" ht="28.8">
       <c r="A150" s="66">
         <v>1</v>
       </c>
@@ -6972,7 +6972,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="151" spans="1:3" ht="27">
+    <row r="151" spans="1:3" ht="28.8">
       <c r="A151" s="66">
         <v>2</v>
       </c>
@@ -6983,7 +6983,7 @@
         <v>265</v>
       </c>
     </row>
-    <row r="152" spans="1:3" ht="27">
+    <row r="152" spans="1:3" ht="28.8">
       <c r="A152" s="66">
         <v>3</v>
       </c>
@@ -7126,19 +7126,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H54"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="15.375" customWidth="1"/>
-    <col min="2" max="2" width="55.75" customWidth="1"/>
+    <col min="1" max="1" width="15.33203125" customWidth="1"/>
+    <col min="2" max="2" width="55.77734375" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
-    <col min="4" max="4" width="9.625" customWidth="1"/>
-    <col min="5" max="5" width="9.25" customWidth="1"/>
-    <col min="6" max="6" width="28.625" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" customWidth="1"/>
+    <col min="5" max="5" width="9.21875" customWidth="1"/>
+    <col min="6" max="6" width="28.6640625" customWidth="1"/>
     <col min="7" max="7" width="19" customWidth="1"/>
-    <col min="8" max="8" width="23.625" customWidth="1"/>
+    <col min="8" max="8" width="23.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="14.25">
+    <row r="1" spans="1:8" ht="15.6">
       <c r="A1" s="110" t="s">
         <v>277</v>
       </c>
@@ -7170,7 +7170,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="25.5">
+    <row r="3" spans="1:8" ht="26.4">
       <c r="A3" s="5">
         <v>0</v>
       </c>
@@ -7190,7 +7190,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="25.5">
+    <row r="4" spans="1:8" ht="26.4">
       <c r="A4" s="5">
         <v>1</v>
       </c>
@@ -7210,7 +7210,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" ht="26.4">
       <c r="A5" s="5">
         <v>2</v>
       </c>
@@ -7270,7 +7270,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" ht="26.4">
       <c r="A8" s="5">
         <v>5</v>
       </c>
@@ -7290,7 +7290,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="9" spans="1:8" ht="25.5">
+    <row r="9" spans="1:8" ht="26.4">
       <c r="A9" s="5">
         <v>6</v>
       </c>
@@ -7310,7 +7310,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="10" spans="1:8" ht="25.5">
+    <row r="10" spans="1:8" ht="39.6">
       <c r="A10" s="5">
         <v>7</v>
       </c>
@@ -7330,7 +7330,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="11" spans="1:8" ht="25.5">
+    <row r="11" spans="1:8" ht="26.4">
       <c r="A11" s="5">
         <v>8</v>
       </c>
@@ -7350,7 +7350,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="25.5">
+    <row r="12" spans="1:8" ht="26.4">
       <c r="A12" s="5">
         <v>9</v>
       </c>
@@ -7370,7 +7370,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="25.5">
+    <row r="13" spans="1:8" ht="26.4">
       <c r="A13" s="5">
         <v>10</v>
       </c>
@@ -7490,7 +7490,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="19" spans="1:8" ht="14.25">
+    <row r="19" spans="1:8" ht="15.6">
       <c r="A19" s="112" t="s">
         <v>309</v>
       </c>
@@ -7842,7 +7842,7 @@
         <v>282</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="14.25">
+    <row r="37" spans="1:8" ht="15.6">
       <c r="A37" s="89"/>
       <c r="B37" s="89"/>
       <c r="C37" s="1"/>
@@ -7948,12 +7948,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:F54"/>
-  <sheetFormatPr defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="23.75" customWidth="1"/>
-    <col min="2" max="2" width="13.75" customWidth="1"/>
-    <col min="3" max="3" width="23.75" customWidth="1"/>
-    <col min="4" max="4" width="22.625" customWidth="1"/>
+    <col min="1" max="1" width="23.77734375" customWidth="1"/>
+    <col min="2" max="2" width="13.77734375" customWidth="1"/>
+    <col min="3" max="3" width="23.77734375" customWidth="1"/>
+    <col min="4" max="4" width="22.6640625" customWidth="1"/>
     <col min="5" max="5" width="25" customWidth="1"/>
   </cols>
   <sheetData>
@@ -8229,7 +8229,7 @@
       </c>
       <c r="F17" s="19"/>
     </row>
-    <row r="18" spans="1:6" ht="89.25">
+    <row r="18" spans="1:6" ht="96.6">
       <c r="A18" s="94">
         <v>10110</v>
       </c>
@@ -8247,7 +8247,7 @@
       </c>
       <c r="F18" s="19"/>
     </row>
-    <row r="19" spans="1:6" ht="24">
+    <row r="19" spans="1:6" ht="36">
       <c r="A19" s="94">
         <v>10111</v>
       </c>
@@ -8265,7 +8265,7 @@
       </c>
       <c r="F19" s="19"/>
     </row>
-    <row r="20" spans="1:6" ht="51">
+    <row r="20" spans="1:6" ht="55.2">
       <c r="A20" s="94">
         <v>10112</v>
       </c>
@@ -8283,7 +8283,7 @@
       </c>
       <c r="F20" s="19"/>
     </row>
-    <row r="21" spans="1:6" ht="24">
+    <row r="21" spans="1:6" ht="36">
       <c r="A21" s="94">
         <v>10118</v>
       </c>
@@ -8301,7 +8301,7 @@
       </c>
       <c r="F21" s="101"/>
     </row>
-    <row r="22" spans="1:6" ht="72">
+    <row r="22" spans="1:6" ht="108">
       <c r="A22" s="94">
         <v>10119</v>
       </c>
@@ -8371,7 +8371,7 @@
       </c>
       <c r="F25" s="101"/>
     </row>
-    <row r="26" spans="1:6" ht="24">
+    <row r="26" spans="1:6" ht="36">
       <c r="A26" s="94">
         <v>10123</v>
       </c>
@@ -8389,7 +8389,7 @@
       </c>
       <c r="F26" s="101"/>
     </row>
-    <row r="27" spans="1:6" ht="25.5">
+    <row r="27" spans="1:6" ht="27.6">
       <c r="A27" s="94">
         <v>10124</v>
       </c>
@@ -8415,7 +8415,7 @@
       <c r="E28" s="93"/>
       <c r="F28" s="40"/>
     </row>
-    <row r="31" spans="1:6" ht="25.5">
+    <row r="31" spans="1:6" ht="43.2">
       <c r="A31" s="11" t="s">
         <v>77</v>
       </c>
@@ -8477,7 +8477,7 @@
       <c r="E34" s="96"/>
       <c r="F34" s="19"/>
     </row>
-    <row r="35" spans="1:6" ht="51">
+    <row r="35" spans="1:6" ht="55.2">
       <c r="A35" s="94">
         <v>15203</v>
       </c>
@@ -8647,7 +8647,7 @@
       </c>
       <c r="F44" s="19"/>
     </row>
-    <row r="45" spans="1:6" ht="24">
+    <row r="45" spans="1:6" ht="36">
       <c r="A45" s="94">
         <v>15213</v>
       </c>
@@ -8665,7 +8665,7 @@
       </c>
       <c r="F45" s="19"/>
     </row>
-    <row r="46" spans="1:6" ht="24">
+    <row r="46" spans="1:6" ht="36">
       <c r="A46" s="94">
         <v>15214</v>
       </c>
@@ -8715,7 +8715,7 @@
       <c r="E48" s="96"/>
       <c r="F48" s="19"/>
     </row>
-    <row r="49" spans="1:6">
+    <row r="49" spans="1:6" ht="24">
       <c r="A49" s="94">
         <v>15217</v>
       </c>
@@ -8821,16 +8821,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="2" width="31.375" customWidth="1"/>
-    <col min="3" max="3" width="22.5" customWidth="1"/>
-    <col min="5" max="5" width="25.625" customWidth="1"/>
-    <col min="6" max="6" width="22.125" customWidth="1"/>
-    <col min="7" max="7" width="20.25" customWidth="1"/>
+    <col min="2" max="2" width="31.33203125" customWidth="1"/>
+    <col min="3" max="3" width="22.44140625" customWidth="1"/>
+    <col min="5" max="5" width="25.6640625" customWidth="1"/>
+    <col min="6" max="6" width="22.109375" customWidth="1"/>
+    <col min="7" max="7" width="20.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="14.25">
+    <row r="1" spans="1:7" ht="15.6">
       <c r="A1" s="110" t="s">
         <v>400</v>
       </c>

</xml_diff>